<commit_message>
Daily recap, matchup updates, learning and research 2026-08-20
</commit_message>
<xml_diff>
--- a/data/k-props/2026-08-20.xlsx
+++ b/data/k-props/2026-08-20.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="77">
   <si>
     <t>date</t>
   </si>
@@ -145,22 +145,34 @@
     <t>lineup_unweighted_30d_posted</t>
   </si>
   <si>
+    <t>U</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>&lt;6</t>
+  </si>
+  <si>
+    <t>Brady Singer</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>&lt;6</t>
-  </si>
-  <si>
-    <t>Brady Singer</t>
-  </si>
-  <si>
     <t>Landen Roupp</t>
   </si>
   <si>
     <t>San Francisco Giants @ Cleveland Guardians</t>
   </si>
   <si>
+    <t>W</t>
+  </si>
+  <si>
     <t>Gavin Williams</t>
+  </si>
+  <si>
+    <t>O</t>
   </si>
   <si>
     <t>&gt;=7</t>
@@ -811,17 +823,23 @@
       <c r="Y2">
         <v>1.0392</v>
       </c>
+      <c r="Z2">
+        <v>4</v>
+      </c>
       <c r="AA2" t="s">
         <v>44</v>
       </c>
+      <c r="AB2">
+        <v>1.01</v>
+      </c>
       <c r="AC2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD2">
         <v>5.51</v>
       </c>
       <c r="AE2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF2">
         <v>0.1811</v>
@@ -831,6 +849,18 @@
       </c>
       <c r="AH2">
         <v>0</v>
+      </c>
+      <c r="AI2">
+        <v>-1.51</v>
+      </c>
+      <c r="AJ2">
+        <v>1.51</v>
+      </c>
+      <c r="AK2">
+        <v>-1.51</v>
+      </c>
+      <c r="AL2">
+        <v>1.51</v>
       </c>
       <c r="AM2">
         <v>5.51</v>
@@ -841,7 +871,7 @@
         <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C3">
         <v>4.5</v>
@@ -912,17 +942,23 @@
       <c r="Y3">
         <v>1.017</v>
       </c>
+      <c r="Z3">
+        <v>3</v>
+      </c>
       <c r="AA3" t="s">
         <v>44</v>
       </c>
+      <c r="AB3">
+        <v>-0.57</v>
+      </c>
       <c r="AC3" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD3">
         <v>3.93</v>
       </c>
       <c r="AE3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF3">
         <v>0.1693</v>
@@ -932,6 +968,18 @@
       </c>
       <c r="AH3">
         <v>0</v>
+      </c>
+      <c r="AI3">
+        <v>-0.93</v>
+      </c>
+      <c r="AJ3">
+        <v>0.93</v>
+      </c>
+      <c r="AK3">
+        <v>-0.93</v>
+      </c>
+      <c r="AL3">
+        <v>0.93</v>
       </c>
       <c r="AM3">
         <v>3.93</v>
@@ -942,7 +990,7 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C4">
         <v>4.5</v>
@@ -954,7 +1002,7 @@
         <v>-139</v>
       </c>
       <c r="F4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G4">
         <v>824395</v>
@@ -1013,17 +1061,23 @@
       <c r="Y4">
         <v>0.8801</v>
       </c>
+      <c r="Z4">
+        <v>2</v>
+      </c>
       <c r="AA4" t="s">
         <v>44</v>
       </c>
+      <c r="AB4">
+        <v>-1.7</v>
+      </c>
       <c r="AC4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD4">
         <v>2.8</v>
       </c>
       <c r="AE4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF4">
         <v>0.1965</v>
@@ -1033,6 +1087,18 @@
       </c>
       <c r="AH4">
         <v>0</v>
+      </c>
+      <c r="AI4">
+        <v>-0.8</v>
+      </c>
+      <c r="AJ4">
+        <v>0.8</v>
+      </c>
+      <c r="AK4">
+        <v>-0.8</v>
+      </c>
+      <c r="AL4">
+        <v>0.8</v>
       </c>
       <c r="AM4">
         <v>2.8</v>
@@ -1043,7 +1109,7 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C5">
         <v>7.5</v>
@@ -1055,7 +1121,7 @@
         <v>-114</v>
       </c>
       <c r="F5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G5">
         <v>824395</v>
@@ -1114,17 +1180,23 @@
       <c r="Y5">
         <v>0.9792</v>
       </c>
+      <c r="Z5">
+        <v>11</v>
+      </c>
       <c r="AA5" t="s">
-        <v>44</v>
+        <v>53</v>
+      </c>
+      <c r="AB5">
+        <v>0.26</v>
       </c>
       <c r="AC5" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD5">
         <v>7.76</v>
       </c>
       <c r="AE5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="AF5">
         <v>0.3506</v>
@@ -1134,6 +1206,18 @@
       </c>
       <c r="AH5">
         <v>0</v>
+      </c>
+      <c r="AI5">
+        <v>3.24</v>
+      </c>
+      <c r="AJ5">
+        <v>3.24</v>
+      </c>
+      <c r="AK5">
+        <v>3.24</v>
+      </c>
+      <c r="AL5">
+        <v>3.24</v>
       </c>
       <c r="AM5">
         <v>7.76</v>
@@ -1144,7 +1228,7 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C6">
         <v>3.5</v>
@@ -1156,7 +1240,7 @@
         <v>110</v>
       </c>
       <c r="F6" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G6">
         <v>822934</v>
@@ -1215,17 +1299,23 @@
       <c r="Y6">
         <v>0.88</v>
       </c>
+      <c r="Z6">
+        <v>7</v>
+      </c>
       <c r="AA6" t="s">
-        <v>44</v>
+        <v>53</v>
+      </c>
+      <c r="AB6">
+        <v>-0.85</v>
       </c>
       <c r="AC6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD6">
         <v>2.65</v>
       </c>
       <c r="AE6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF6">
         <v>0.1883</v>
@@ -1235,6 +1325,18 @@
       </c>
       <c r="AH6">
         <v>0</v>
+      </c>
+      <c r="AI6">
+        <v>4.35</v>
+      </c>
+      <c r="AJ6">
+        <v>4.35</v>
+      </c>
+      <c r="AK6">
+        <v>4.35</v>
+      </c>
+      <c r="AL6">
+        <v>4.35</v>
       </c>
       <c r="AM6">
         <v>2.65</v>
@@ -1245,7 +1347,7 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C7">
         <v>5.5</v>
@@ -1257,7 +1359,7 @@
         <v>-134</v>
       </c>
       <c r="F7" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G7">
         <v>822934</v>
@@ -1316,17 +1418,23 @@
       <c r="Y7">
         <v>0.9434</v>
       </c>
+      <c r="Z7">
+        <v>8</v>
+      </c>
       <c r="AA7" t="s">
-        <v>44</v>
+        <v>53</v>
+      </c>
+      <c r="AB7">
+        <v>-1.16</v>
       </c>
       <c r="AC7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD7">
         <v>4.34</v>
       </c>
       <c r="AE7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF7">
         <v>0.3069</v>
@@ -1336,6 +1444,18 @@
       </c>
       <c r="AH7">
         <v>0</v>
+      </c>
+      <c r="AI7">
+        <v>3.66</v>
+      </c>
+      <c r="AJ7">
+        <v>3.66</v>
+      </c>
+      <c r="AK7">
+        <v>3.66</v>
+      </c>
+      <c r="AL7">
+        <v>3.66</v>
       </c>
       <c r="AM7">
         <v>4.34</v>
@@ -1346,7 +1466,7 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C8">
         <v>4.5</v>
@@ -1358,7 +1478,7 @@
         <v>116</v>
       </c>
       <c r="F8" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G8">
         <v>824074</v>
@@ -1417,17 +1537,23 @@
       <c r="Y8">
         <v>0.88</v>
       </c>
+      <c r="Z8">
+        <v>3</v>
+      </c>
       <c r="AA8" t="s">
         <v>44</v>
       </c>
+      <c r="AB8">
+        <v>-0.07</v>
+      </c>
       <c r="AC8" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD8">
         <v>4.43</v>
       </c>
       <c r="AE8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF8">
         <v>0.2397</v>
@@ -1437,6 +1563,18 @@
       </c>
       <c r="AH8">
         <v>0</v>
+      </c>
+      <c r="AI8">
+        <v>-1.43</v>
+      </c>
+      <c r="AJ8">
+        <v>1.43</v>
+      </c>
+      <c r="AK8">
+        <v>-1.43</v>
+      </c>
+      <c r="AL8">
+        <v>1.43</v>
       </c>
       <c r="AM8">
         <v>4.43</v>
@@ -1447,7 +1585,7 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C9">
         <v>3.5</v>
@@ -1459,7 +1597,7 @@
         <v>-149</v>
       </c>
       <c r="F9" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G9">
         <v>824074</v>
@@ -1518,17 +1656,23 @@
       <c r="Y9">
         <v>1.0024</v>
       </c>
+      <c r="Z9">
+        <v>4</v>
+      </c>
       <c r="AA9" t="s">
-        <v>44</v>
+        <v>53</v>
+      </c>
+      <c r="AB9">
+        <v>-0.38</v>
       </c>
       <c r="AC9" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD9">
         <v>3.12</v>
       </c>
       <c r="AE9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF9">
         <v>0.1538</v>
@@ -1538,6 +1682,18 @@
       </c>
       <c r="AH9">
         <v>0</v>
+      </c>
+      <c r="AI9">
+        <v>0.88</v>
+      </c>
+      <c r="AJ9">
+        <v>0.88</v>
+      </c>
+      <c r="AK9">
+        <v>0.88</v>
+      </c>
+      <c r="AL9">
+        <v>0.88</v>
       </c>
       <c r="AM9">
         <v>3.12</v>
@@ -1548,7 +1704,7 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C10">
         <v>4.5</v>
@@ -1560,7 +1716,7 @@
         <v>-135</v>
       </c>
       <c r="F10" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G10">
         <v>824589</v>
@@ -1619,17 +1775,23 @@
       <c r="Y10">
         <v>1.0597</v>
       </c>
+      <c r="Z10">
+        <v>3</v>
+      </c>
       <c r="AA10" t="s">
         <v>44</v>
       </c>
+      <c r="AB10">
+        <v>-0.19</v>
+      </c>
       <c r="AC10" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD10">
         <v>4.31</v>
       </c>
       <c r="AE10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF10">
         <v>0.1785</v>
@@ -1639,6 +1801,18 @@
       </c>
       <c r="AH10">
         <v>0</v>
+      </c>
+      <c r="AI10">
+        <v>-1.31</v>
+      </c>
+      <c r="AJ10">
+        <v>1.31</v>
+      </c>
+      <c r="AK10">
+        <v>-1.31</v>
+      </c>
+      <c r="AL10">
+        <v>1.31</v>
       </c>
       <c r="AM10">
         <v>4.31</v>
@@ -1649,7 +1823,7 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C11">
         <v>4.5</v>
@@ -1661,7 +1835,7 @@
         <v>-130</v>
       </c>
       <c r="F11" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G11">
         <v>824589</v>
@@ -1720,17 +1894,23 @@
       <c r="Y11">
         <v>0.9771</v>
       </c>
+      <c r="Z11">
+        <v>6</v>
+      </c>
       <c r="AA11" t="s">
-        <v>44</v>
+        <v>53</v>
+      </c>
+      <c r="AB11">
+        <v>0.31</v>
       </c>
       <c r="AC11" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD11">
         <v>4.81</v>
       </c>
       <c r="AE11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF11">
         <v>0.1895</v>
@@ -1740,6 +1920,18 @@
       </c>
       <c r="AH11">
         <v>0</v>
+      </c>
+      <c r="AI11">
+        <v>1.19</v>
+      </c>
+      <c r="AJ11">
+        <v>1.19</v>
+      </c>
+      <c r="AK11">
+        <v>1.19</v>
+      </c>
+      <c r="AL11">
+        <v>1.19</v>
       </c>
       <c r="AM11">
         <v>4.81</v>
@@ -1750,7 +1942,7 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C12">
         <v>4.5</v>
@@ -1762,7 +1954,7 @@
         <v>112</v>
       </c>
       <c r="F12" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="G12">
         <v>823747</v>
@@ -1821,17 +2013,23 @@
       <c r="Y12">
         <v>1.0224</v>
       </c>
+      <c r="Z12">
+        <v>3</v>
+      </c>
       <c r="AA12" t="s">
         <v>44</v>
       </c>
+      <c r="AB12">
+        <v>0.16</v>
+      </c>
       <c r="AC12" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD12">
         <v>4.66</v>
       </c>
       <c r="AE12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF12">
         <v>0.1705</v>
@@ -1841,6 +2039,18 @@
       </c>
       <c r="AH12">
         <v>0</v>
+      </c>
+      <c r="AI12">
+        <v>-1.66</v>
+      </c>
+      <c r="AJ12">
+        <v>1.66</v>
+      </c>
+      <c r="AK12">
+        <v>-1.66</v>
+      </c>
+      <c r="AL12">
+        <v>1.66</v>
       </c>
       <c r="AM12">
         <v>4.66</v>
@@ -1851,7 +2061,7 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C13">
         <v>5.5</v>
@@ -1863,7 +2073,7 @@
         <v>-144</v>
       </c>
       <c r="F13" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="G13">
         <v>823747</v>
@@ -1922,17 +2132,23 @@
       <c r="Y13">
         <v>0.9308</v>
       </c>
+      <c r="Z13">
+        <v>4</v>
+      </c>
       <c r="AA13" t="s">
         <v>44</v>
       </c>
+      <c r="AB13">
+        <v>-1.31</v>
+      </c>
       <c r="AC13" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD13">
         <v>4.19</v>
       </c>
       <c r="AE13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF13">
         <v>0.2131</v>
@@ -1942,6 +2158,18 @@
       </c>
       <c r="AH13">
         <v>0</v>
+      </c>
+      <c r="AI13">
+        <v>-0.19</v>
+      </c>
+      <c r="AJ13">
+        <v>0.19</v>
+      </c>
+      <c r="AK13">
+        <v>-0.19</v>
+      </c>
+      <c r="AL13">
+        <v>0.19</v>
       </c>
       <c r="AM13">
         <v>4.19</v>
@@ -1952,7 +2180,7 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C14">
         <v>6.5</v>
@@ -1964,7 +2192,7 @@
         <v>-102</v>
       </c>
       <c r="F14" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G14">
         <v>824802</v>
@@ -2023,17 +2251,23 @@
       <c r="Y14">
         <v>1.0903</v>
       </c>
+      <c r="Z14">
+        <v>8</v>
+      </c>
       <c r="AA14" t="s">
-        <v>44</v>
+        <v>53</v>
+      </c>
+      <c r="AB14">
+        <v>1.79</v>
       </c>
       <c r="AC14" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD14">
         <v>8.29</v>
       </c>
       <c r="AE14" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="AF14">
         <v>0.2759</v>
@@ -2043,6 +2277,18 @@
       </c>
       <c r="AH14">
         <v>0</v>
+      </c>
+      <c r="AI14">
+        <v>-0.29</v>
+      </c>
+      <c r="AJ14">
+        <v>0.29</v>
+      </c>
+      <c r="AK14">
+        <v>-0.29</v>
+      </c>
+      <c r="AL14">
+        <v>0.29</v>
       </c>
       <c r="AM14">
         <v>8.29</v>
@@ -2053,7 +2299,7 @@
         <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C15">
         <v>5.5</v>
@@ -2065,7 +2311,7 @@
         <v>112</v>
       </c>
       <c r="F15" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G15">
         <v>824802</v>
@@ -2124,17 +2370,23 @@
       <c r="Y15">
         <v>1.0556</v>
       </c>
+      <c r="Z15">
+        <v>5</v>
+      </c>
       <c r="AA15" t="s">
         <v>44</v>
       </c>
+      <c r="AB15">
+        <v>0.76</v>
+      </c>
       <c r="AC15" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD15">
         <v>6.08</v>
       </c>
       <c r="AE15" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="AF15">
         <v>0.2017</v>
@@ -2144,6 +2396,18 @@
       </c>
       <c r="AH15">
         <v>0.18</v>
+      </c>
+      <c r="AI15">
+        <v>-1.08</v>
+      </c>
+      <c r="AJ15">
+        <v>1.08</v>
+      </c>
+      <c r="AK15">
+        <v>-1.26</v>
+      </c>
+      <c r="AL15">
+        <v>1.26</v>
       </c>
       <c r="AM15">
         <v>6.26</v>
@@ -2154,7 +2418,7 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C16">
         <v>4.5</v>
@@ -2166,7 +2430,7 @@
         <v>-124</v>
       </c>
       <c r="F16" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G16">
         <v>822861</v>
@@ -2225,17 +2489,23 @@
       <c r="Y16">
         <v>1.0527</v>
       </c>
+      <c r="Z16">
+        <v>5</v>
+      </c>
       <c r="AA16" t="s">
-        <v>44</v>
+        <v>53</v>
+      </c>
+      <c r="AB16">
+        <v>0.47</v>
       </c>
       <c r="AC16" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD16">
         <v>4.97</v>
       </c>
       <c r="AE16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF16">
         <v>0.1902</v>
@@ -2245,6 +2515,18 @@
       </c>
       <c r="AH16">
         <v>0</v>
+      </c>
+      <c r="AI16">
+        <v>0.03</v>
+      </c>
+      <c r="AJ16">
+        <v>0.03</v>
+      </c>
+      <c r="AK16">
+        <v>0.03</v>
+      </c>
+      <c r="AL16">
+        <v>0.03</v>
       </c>
       <c r="AM16">
         <v>4.97</v>
@@ -2255,7 +2537,7 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C17">
         <v>6.5</v>
@@ -2267,7 +2549,7 @@
         <v>-140</v>
       </c>
       <c r="F17" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G17">
         <v>822861</v>
@@ -2326,17 +2608,23 @@
       <c r="Y17">
         <v>1.0365</v>
       </c>
+      <c r="Z17">
+        <v>10</v>
+      </c>
       <c r="AA17" t="s">
-        <v>44</v>
+        <v>53</v>
+      </c>
+      <c r="AB17">
+        <v>-0.08</v>
       </c>
       <c r="AC17" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD17">
         <v>6.24</v>
       </c>
       <c r="AE17" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="AF17">
         <v>0.2829</v>
@@ -2346,6 +2634,18 @@
       </c>
       <c r="AH17">
         <v>0.18</v>
+      </c>
+      <c r="AI17">
+        <v>3.76</v>
+      </c>
+      <c r="AJ17">
+        <v>3.76</v>
+      </c>
+      <c r="AK17">
+        <v>3.58</v>
+      </c>
+      <c r="AL17">
+        <v>3.58</v>
       </c>
       <c r="AM17">
         <v>6.42</v>
@@ -2356,7 +2656,7 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C18">
         <v>4.5</v>
@@ -2368,7 +2668,7 @@
         <v>104</v>
       </c>
       <c r="F18" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G18">
         <v>824153</v>
@@ -2427,17 +2727,23 @@
       <c r="Y18">
         <v>0.9281</v>
       </c>
+      <c r="Z18">
+        <v>6</v>
+      </c>
       <c r="AA18" t="s">
-        <v>44</v>
+        <v>53</v>
+      </c>
+      <c r="AB18">
+        <v>-0.6</v>
       </c>
       <c r="AC18" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD18">
         <v>3.9</v>
       </c>
       <c r="AE18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF18">
         <v>0.2264</v>
@@ -2447,6 +2753,18 @@
       </c>
       <c r="AH18">
         <v>0</v>
+      </c>
+      <c r="AI18">
+        <v>2.1</v>
+      </c>
+      <c r="AJ18">
+        <v>2.1</v>
+      </c>
+      <c r="AK18">
+        <v>2.1</v>
+      </c>
+      <c r="AL18">
+        <v>2.1</v>
       </c>
       <c r="AM18">
         <v>3.9</v>
@@ -2457,7 +2775,7 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C19">
         <v>5.5</v>
@@ -2469,7 +2787,7 @@
         <v>-114</v>
       </c>
       <c r="F19" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G19">
         <v>824153</v>
@@ -2528,17 +2846,23 @@
       <c r="Y19">
         <v>0.99</v>
       </c>
+      <c r="Z19">
+        <v>3</v>
+      </c>
       <c r="AA19" t="s">
         <v>44</v>
       </c>
+      <c r="AB19">
+        <v>-0.29</v>
+      </c>
       <c r="AC19" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD19">
         <v>5.21</v>
       </c>
       <c r="AE19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF19">
         <v>0.2329</v>
@@ -2548,6 +2872,18 @@
       </c>
       <c r="AH19">
         <v>0</v>
+      </c>
+      <c r="AI19">
+        <v>-2.21</v>
+      </c>
+      <c r="AJ19">
+        <v>2.21</v>
+      </c>
+      <c r="AK19">
+        <v>-2.21</v>
+      </c>
+      <c r="AL19">
+        <v>2.21</v>
       </c>
       <c r="AM19">
         <v>5.21</v>

</xml_diff>